<commit_message>
Pre Market Mon 2026-07-06
</commit_message>
<xml_diff>
--- a/market-prep/Pre Market 2026-07-06.xlsx
+++ b/market-prep/Pre Market 2026-07-06.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,7 +459,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>7466,24</t>
+          <t>7483,24</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -476,7 +476,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>29208,97</t>
+          <t>29329,21</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -493,7 +493,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2996,10</t>
+          <t>2996,11</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -510,7 +510,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>52776,22</t>
+          <t>52900,07</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>4119,86</t>
+          <t>4122,37</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>60,83</t>
+          <t>60,91</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1621,33</t>
+          <t>1621,50</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>71,61</t>
+          <t>71,80</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>61343,11</t>
+          <t>61460,41</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1697,19</t>
+          <t>1701,76</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -724,7 +724,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-0,72%</t>
+          <t>-2,65%</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -750,41 +750,28 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>7460,11</t>
+          <t>7483,24</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Neg Corr</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Divergent</t>
-        </is>
-      </c>
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr"/>
-      <c r="B25" t="inlineStr"/>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Fear Greed Index</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
       <c r="C25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Fear Greed Index</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>